<commit_message>
Added Input Lists for Output Files
Added created PDF and Zip based on input list of characters.
</commit_message>
<xml_diff>
--- a/input/character_update_august_2026.xlsx
+++ b/input/character_update_august_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brad/Documents/GitHub/crop_mcp_cards/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6291C0B-27BF-8245-94AA-9326015AFFF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{609E9689-B60D-6640-8068-FCD38F9DCA63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1180" yWindow="660" windowWidth="29060" windowHeight="18980" xr2:uid="{3BD2E35C-BAB5-3F4C-BF56-002E203FB5BC}"/>
+    <workbookView xWindow="1280" yWindow="660" windowWidth="28960" windowHeight="18980" xr2:uid="{3BD2E35C-BAB5-3F4C-BF56-002E203FB5BC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="465">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="693" uniqueCount="468">
   <si>
     <t>01620101</t>
   </si>
@@ -1361,12 +1361,6 @@
     <t>King T'Challa</t>
   </si>
   <si>
-    <t>T0000001</t>
-  </si>
-  <si>
-    <t>Jubilee</t>
-  </si>
-  <si>
     <t>20130101</t>
   </si>
   <si>
@@ -1434,6 +1428,21 @@
   </si>
   <si>
     <t>File</t>
+  </si>
+  <si>
+    <t>Update Type</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Health</t>
+  </si>
+  <si>
+    <t>Rules</t>
+  </si>
+  <si>
+    <t>Peerless</t>
   </si>
 </sst>
 </file>
@@ -1485,7 +1494,10 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="8">
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
     <dxf>
       <protection locked="0" hidden="0"/>
     </dxf>
@@ -1521,23 +1533,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E1E3FA1E-FC30-AC41-815B-A3E7F9829415}" name="Table1" displayName="Table1" ref="A1:K231" totalsRowShown="0" headerRowDxfId="6">
-  <autoFilter ref="A1:K231" xr:uid="{E1E3FA1E-FC30-AC41-815B-A3E7F9829415}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E1E3FA1E-FC30-AC41-815B-A3E7F9829415}" name="Table1" displayName="Table1" ref="A1:L230" totalsRowShown="0" headerRowDxfId="7">
+  <autoFilter ref="A1:L230" xr:uid="{E1E3FA1E-FC30-AC41-815B-A3E7F9829415}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J230">
     <sortCondition ref="B1:B230"/>
   </sortState>
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{18E46103-64C1-6A4D-BAE4-D926501D8281}" name="MCT Code" dataDxfId="5"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{18E46103-64C1-6A4D-BAE4-D926501D8281}" name="MCT Code" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{571D3DAC-1677-914B-AFC7-BB1B0A7D42A4}" name="Character Name"/>
     <tableColumn id="3" xr3:uid="{35C6C37F-0418-6D4D-93AE-AA3759287D39}" name="Threat"/>
     <tableColumn id="4" xr3:uid="{36738C16-1A81-D84F-ACAB-88BB42541BC4}" name="Current Front"/>
     <tableColumn id="5" xr3:uid="{E708D589-BDB3-CE43-ADE3-2633E7337332}" name="Current Back"/>
     <tableColumn id="6" xr3:uid="{1709A50E-52CC-6440-B627-D53155B54710}" name="Current Extra Power"/>
-    <tableColumn id="7" xr3:uid="{64A16CF9-664E-0843-898F-C278F07E409C}" name="Page Number" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{C3DD3B62-707D-484A-B7C4-F65A85D1F048}" name="Updated Front" dataDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{9CF1A1F3-A863-B14E-A8A3-55012E20E2F8}" name="Updated Back" dataDxfId="2"/>
-    <tableColumn id="10" xr3:uid="{6E4A6AF0-64C8-6747-A7CE-104AA5B75FED}" name="Updated Extra Power" dataDxfId="1"/>
-    <tableColumn id="11" xr3:uid="{EFE7CA5B-10E7-B04E-9D9E-CFF9B4B9C2AA}" name="File" dataDxfId="0"/>
+    <tableColumn id="7" xr3:uid="{64A16CF9-664E-0843-898F-C278F07E409C}" name="Page Number" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{C3DD3B62-707D-484A-B7C4-F65A85D1F048}" name="Updated Front" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{9CF1A1F3-A863-B14E-A8A3-55012E20E2F8}" name="Updated Back" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{6E4A6AF0-64C8-6747-A7CE-104AA5B75FED}" name="Updated Extra Power" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{EFE7CA5B-10E7-B04E-9D9E-CFF9B4B9C2AA}" name="File" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{04E36717-29D7-C847-9743-DF3222FDE485}" name="Update Type" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1860,7 +1873,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17D228EF-F196-D04E-A0A4-FC2E940450C5}">
-  <dimension ref="A1:K231"/>
+  <dimension ref="A1:L230"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.83203125" style="1" customWidth="1"/>
@@ -1870,42 +1883,45 @@
     <col min="7" max="10" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="3" customFormat="1" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" s="3" customFormat="1" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>445</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>446</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>447</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>448</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="G1" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>449</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>450</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>444</v>
-      </c>
-      <c r="H1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>451</v>
       </c>
-      <c r="I1" s="3" t="s">
-        <v>452</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>453</v>
-      </c>
       <c r="K1" s="3" t="s">
-        <v>464</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+        <v>462</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1933,8 +1949,11 @@
       <c r="K2" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L2" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -1962,8 +1981,11 @@
       <c r="K3" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L3" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -1995,8 +2017,11 @@
       <c r="K4" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L4" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -2028,8 +2053,11 @@
       <c r="K5" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L5" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
@@ -2063,8 +2091,11 @@
       <c r="K6" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L6" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>45</v>
       </c>
@@ -2096,8 +2127,11 @@
       <c r="K7" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L7" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>10</v>
       </c>
@@ -2131,13 +2165,16 @@
       <c r="K8" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L8" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="C9">
         <v>3</v>
@@ -2164,10 +2201,13 @@
       <c r="K9" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L9" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="G10" s="4">
         <v>9</v>
@@ -2178,8 +2218,11 @@
       <c r="K10" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L10" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>47</v>
       </c>
@@ -2207,8 +2250,11 @@
       <c r="K11" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L11" s="4" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>49</v>
       </c>
@@ -2240,8 +2286,11 @@
       <c r="K12" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L12" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>13</v>
       </c>
@@ -2273,8 +2322,11 @@
       <c r="K13" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L13" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>15</v>
       </c>
@@ -2306,8 +2358,11 @@
       <c r="K14" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L14" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>17</v>
       </c>
@@ -2339,8 +2394,11 @@
       <c r="K15" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L15" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>19</v>
       </c>
@@ -2372,8 +2430,11 @@
       <c r="K16" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L16" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>21</v>
       </c>
@@ -2405,8 +2466,11 @@
       <c r="K17" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L17" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>23</v>
       </c>
@@ -2438,8 +2502,11 @@
       <c r="K18" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L18" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>25</v>
       </c>
@@ -2467,8 +2534,11 @@
       <c r="K19" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L19" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>27</v>
       </c>
@@ -2502,8 +2572,11 @@
       <c r="K20" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L20" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>29</v>
       </c>
@@ -2535,8 +2608,11 @@
       <c r="K21" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L21" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>31</v>
       </c>
@@ -2570,8 +2646,11 @@
       <c r="K22" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L22" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>33</v>
       </c>
@@ -2599,8 +2678,11 @@
       <c r="K23" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L23" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>35</v>
       </c>
@@ -2632,8 +2714,11 @@
       <c r="K24" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L24" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>37</v>
       </c>
@@ -2665,8 +2750,11 @@
       <c r="K25" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L25" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>434</v>
       </c>
@@ -2698,8 +2786,11 @@
       <c r="K26" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L26" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>39</v>
       </c>
@@ -2731,8 +2822,11 @@
       <c r="K27" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L27" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>41</v>
       </c>
@@ -2760,8 +2854,11 @@
       <c r="K28" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L28" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>43</v>
       </c>
@@ -2789,8 +2886,11 @@
       <c r="K29" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L29" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>71</v>
       </c>
@@ -2822,8 +2922,11 @@
       <c r="K30" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L30" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>73</v>
       </c>
@@ -2851,8 +2954,11 @@
       <c r="K31" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L31" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>75</v>
       </c>
@@ -2880,8 +2986,11 @@
       <c r="K32" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L32" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>77</v>
       </c>
@@ -2909,8 +3018,11 @@
       <c r="K33" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L33" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>79</v>
       </c>
@@ -2944,8 +3056,11 @@
       <c r="K34" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L34" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>81</v>
       </c>
@@ -2977,8 +3092,11 @@
       <c r="K35" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L35" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>83</v>
       </c>
@@ -3010,8 +3128,11 @@
       <c r="K36" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L36" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>85</v>
       </c>
@@ -3043,8 +3164,11 @@
       <c r="K37" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L37" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>87</v>
       </c>
@@ -3076,8 +3200,11 @@
       <c r="K38" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L38" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>89</v>
       </c>
@@ -3109,10 +3236,13 @@
       <c r="K39" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L39" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B40" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="G40" s="4">
         <v>39</v>
@@ -3123,8 +3253,11 @@
       <c r="K40" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L40" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>91</v>
       </c>
@@ -3152,8 +3285,11 @@
       <c r="K41" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L41" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>93</v>
       </c>
@@ -3187,8 +3323,11 @@
       <c r="K42" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L42" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>95</v>
       </c>
@@ -3220,8 +3359,11 @@
       <c r="K43" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L43" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>97</v>
       </c>
@@ -3253,8 +3395,11 @@
       <c r="K44" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L44" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>99</v>
       </c>
@@ -3286,8 +3431,11 @@
       <c r="K45" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L45" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>432</v>
       </c>
@@ -3315,8 +3463,11 @@
       <c r="K46" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L46" s="4" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>101</v>
       </c>
@@ -3344,8 +3495,11 @@
       <c r="K47" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L47" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>103</v>
       </c>
@@ -3373,8 +3527,11 @@
       <c r="K48" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L48" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>105</v>
       </c>
@@ -3402,8 +3559,11 @@
       <c r="K49" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L49" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>107</v>
       </c>
@@ -3435,8 +3595,11 @@
       <c r="K50" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L50" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>109</v>
       </c>
@@ -3468,8 +3631,11 @@
       <c r="K51" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L51" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>111</v>
       </c>
@@ -3501,8 +3667,11 @@
       <c r="K52" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L52" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
         <v>113</v>
       </c>
@@ -3534,8 +3703,11 @@
       <c r="K53" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L53" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
         <v>115</v>
       </c>
@@ -3567,8 +3739,11 @@
       <c r="K54" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L54" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>117</v>
       </c>
@@ -3600,8 +3775,11 @@
       <c r="K55" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L55" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
         <v>119</v>
       </c>
@@ -3633,8 +3811,11 @@
       <c r="K56" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L56" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
         <v>51</v>
       </c>
@@ -3666,8 +3847,11 @@
       <c r="K57" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L57" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
         <v>121</v>
       </c>
@@ -3701,8 +3885,11 @@
       <c r="K58" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L58" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>123</v>
       </c>
@@ -3730,8 +3917,11 @@
       <c r="K59" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L59" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
         <v>125</v>
       </c>
@@ -3763,8 +3953,11 @@
       <c r="K60" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L60" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
         <v>127</v>
       </c>
@@ -3792,8 +3985,11 @@
       <c r="K61" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L61" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
         <v>129</v>
       </c>
@@ -3821,8 +4017,11 @@
       <c r="K62" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L62" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
         <v>131</v>
       </c>
@@ -3850,8 +4049,11 @@
       <c r="K63" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L63" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
         <v>133</v>
       </c>
@@ -3883,8 +4085,11 @@
       <c r="K64" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L64" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
         <v>135</v>
       </c>
@@ -3916,8 +4121,11 @@
       <c r="K65" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L65" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
         <v>137</v>
       </c>
@@ -3949,8 +4157,11 @@
       <c r="K66" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L66" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
         <v>139</v>
       </c>
@@ -3982,8 +4193,11 @@
       <c r="K67" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L67" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
         <v>141</v>
       </c>
@@ -4015,8 +4229,11 @@
       <c r="K68" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L68" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
         <v>143</v>
       </c>
@@ -4048,10 +4265,13 @@
       <c r="K69" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L69" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B70" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="G70" s="4">
         <v>69</v>
@@ -4062,8 +4282,11 @@
       <c r="K70" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L70" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
         <v>145</v>
       </c>
@@ -4097,8 +4320,11 @@
       <c r="K71" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L71" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
         <v>147</v>
       </c>
@@ -4132,8 +4358,11 @@
       <c r="K72" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L72" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
         <v>149</v>
       </c>
@@ -4165,8 +4394,11 @@
       <c r="K73" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L73" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
         <v>151</v>
       </c>
@@ -4198,8 +4430,11 @@
       <c r="K74" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L74" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
         <v>153</v>
       </c>
@@ -4231,8 +4466,11 @@
       <c r="K75" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L75" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
         <v>155</v>
       </c>
@@ -4260,8 +4498,11 @@
       <c r="K76" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L76" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
         <v>157</v>
       </c>
@@ -4293,13 +4534,16 @@
       <c r="K77" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L77" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="B78" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="C78">
         <v>6</v>
@@ -4322,8 +4566,11 @@
       <c r="K78" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L78" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
         <v>159</v>
       </c>
@@ -4351,8 +4598,11 @@
       <c r="K79" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L79" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="80" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
         <v>161</v>
       </c>
@@ -4384,8 +4634,11 @@
       <c r="K80" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L80" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
         <v>163</v>
       </c>
@@ -4413,8 +4666,11 @@
       <c r="K81" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L81" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
         <v>165</v>
       </c>
@@ -4446,8 +4702,11 @@
       <c r="K82" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L82" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
         <v>167</v>
       </c>
@@ -4479,8 +4738,11 @@
       <c r="K83" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L83" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
         <v>169</v>
       </c>
@@ -4508,8 +4770,11 @@
       <c r="K84" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L84" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
         <v>171</v>
       </c>
@@ -4541,8 +4806,11 @@
       <c r="K85" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L85" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A86" s="1" t="s">
         <v>173</v>
       </c>
@@ -4576,8 +4844,11 @@
       <c r="K86" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L86" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="s">
         <v>175</v>
       </c>
@@ -4605,13 +4876,16 @@
       <c r="K87" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L87" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="88" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A88" s="1" t="s">
         <v>177</v>
       </c>
       <c r="B88" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="C88">
         <v>3</v>
@@ -4638,10 +4912,13 @@
       <c r="K88" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L88" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="89" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B89" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="G89" s="4">
         <v>11</v>
@@ -4652,8 +4929,11 @@
       <c r="K89" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L89" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="90" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
         <v>422</v>
       </c>
@@ -4678,8 +4958,11 @@
       <c r="K90" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L90" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="91" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A91" s="1" t="s">
         <v>178</v>
       </c>
@@ -4713,8 +4996,11 @@
       <c r="K91" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L91" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="92" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="s">
         <v>180</v>
       </c>
@@ -4746,8 +5032,11 @@
       <c r="K92" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L92" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="93" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
         <v>182</v>
       </c>
@@ -4779,8 +5068,11 @@
       <c r="K93" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L93" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="94" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
         <v>184</v>
       </c>
@@ -4814,8 +5106,11 @@
       <c r="K94" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L94" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="95" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="s">
         <v>186</v>
       </c>
@@ -4843,8 +5138,11 @@
       <c r="K95" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L95" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="96" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="s">
         <v>188</v>
       </c>
@@ -4876,8 +5174,11 @@
       <c r="K96" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L96" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="97" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
         <v>190</v>
       </c>
@@ -4905,8 +5206,11 @@
       <c r="K97" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L97" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="98" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
         <v>192</v>
       </c>
@@ -4940,8 +5244,11 @@
       <c r="K98" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L98" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="99" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
         <v>194</v>
       </c>
@@ -4969,8 +5276,11 @@
       <c r="K99" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L99" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="100" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A100" s="1" t="s">
         <v>196</v>
       </c>
@@ -5002,8 +5312,11 @@
       <c r="K100" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L100" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="101" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A101" s="1" t="s">
         <v>198</v>
       </c>
@@ -5031,8 +5344,11 @@
       <c r="K101" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L101" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="102" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A102" s="1" t="s">
         <v>200</v>
       </c>
@@ -5064,8 +5380,11 @@
       <c r="K102" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L102" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="103" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A103" s="1" t="s">
         <v>436</v>
       </c>
@@ -5097,8 +5416,11 @@
       <c r="K103" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L103" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="104" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A104" s="1" t="s">
         <v>202</v>
       </c>
@@ -5126,8 +5448,11 @@
       <c r="K104" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L104" s="4" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="105" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A105" s="1" t="s">
         <v>438</v>
       </c>
@@ -5155,8 +5480,11 @@
       <c r="K105" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L105" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="106" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A106" s="1" t="s">
         <v>204</v>
       </c>
@@ -5184,8 +5512,11 @@
       <c r="K106" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L106" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="107" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A107" s="1" t="s">
         <v>206</v>
       </c>
@@ -5217,8 +5548,11 @@
       <c r="K107" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L107" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="108" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A108" s="1" t="s">
         <v>208</v>
       </c>
@@ -5250,8 +5584,11 @@
       <c r="K108" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L108" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="109" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="s">
         <v>210</v>
       </c>
@@ -5283,8 +5620,11 @@
       <c r="K109" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L109" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="110" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A110" s="1" t="s">
         <v>212</v>
       </c>
@@ -5318,8 +5658,11 @@
       <c r="K110" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L110" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="111" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A111" s="1" t="s">
         <v>214</v>
       </c>
@@ -5347,8 +5690,11 @@
       <c r="K111" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L111" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="112" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A112" s="1" t="s">
         <v>216</v>
       </c>
@@ -5380,8 +5726,11 @@
       <c r="K112" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L112" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="113" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A113" s="1" t="s">
         <v>428</v>
       </c>
@@ -5413,8 +5762,11 @@
       <c r="K113" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L113" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="114" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A114" s="1" t="s">
         <v>218</v>
       </c>
@@ -5448,8 +5800,11 @@
       <c r="K114" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L114" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="115" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A115" s="1" t="s">
         <v>220</v>
       </c>
@@ -5477,8 +5832,11 @@
       <c r="K115" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L115" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="116" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A116" s="1" t="s">
         <v>222</v>
       </c>
@@ -5506,8 +5864,11 @@
       <c r="K116" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L116" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="117" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A117" s="1" t="s">
         <v>230</v>
       </c>
@@ -5539,8 +5900,11 @@
       <c r="K117" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L117" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="118" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A118" s="1" t="s">
         <v>232</v>
       </c>
@@ -5572,8 +5936,11 @@
       <c r="K118" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L118" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="119" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A119" s="1" t="s">
         <v>53</v>
       </c>
@@ -5605,8 +5972,11 @@
       <c r="K119" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L119" s="4" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="120" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A120" s="1" t="s">
         <v>234</v>
       </c>
@@ -5634,8 +6004,11 @@
       <c r="K120" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L120" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="121" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A121" s="1" t="s">
         <v>55</v>
       </c>
@@ -5667,8 +6040,11 @@
       <c r="K121" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L121" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="122" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A122" s="1" t="s">
         <v>57</v>
       </c>
@@ -5700,8 +6076,11 @@
       <c r="K122" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L122" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="123" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A123" s="1" t="s">
         <v>224</v>
       </c>
@@ -5733,8 +6112,11 @@
       <c r="K123" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L123" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="124" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A124" s="1" t="s">
         <v>236</v>
       </c>
@@ -5766,8 +6148,11 @@
       <c r="K124" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L124" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="125" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A125" s="1" t="s">
         <v>238</v>
       </c>
@@ -5795,8 +6180,11 @@
       <c r="K125" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L125" s="4" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="126" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A126" s="1" t="s">
         <v>240</v>
       </c>
@@ -5828,8 +6216,11 @@
       <c r="K126" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L126" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="127" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A127" s="1" t="s">
         <v>226</v>
       </c>
@@ -5861,8 +6252,11 @@
       <c r="K127" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L127" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="128" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A128" s="1" t="s">
         <v>228</v>
       </c>
@@ -5894,8 +6288,11 @@
       <c r="K128" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L128" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="129" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A129" s="1" t="s">
         <v>242</v>
       </c>
@@ -5927,8 +6324,11 @@
       <c r="K129" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L129" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="130" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A130" s="1" t="s">
         <v>244</v>
       </c>
@@ -5956,13 +6356,16 @@
       <c r="K130" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L130" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="131" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A131" s="1" t="s">
         <v>246</v>
       </c>
       <c r="B131" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="C131">
         <v>3</v>
@@ -5989,10 +6392,13 @@
       <c r="K131" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L131" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="132" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B132" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="G132" s="4">
         <v>54</v>
@@ -6003,8 +6409,11 @@
       <c r="K132" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L132" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="133" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A133" s="1" t="s">
         <v>247</v>
       </c>
@@ -6036,8 +6445,11 @@
       <c r="K133" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L133" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="134" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A134" s="1" t="s">
         <v>249</v>
       </c>
@@ -6069,8 +6481,11 @@
       <c r="K134" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L134" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="135" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A135" s="1" t="s">
         <v>253</v>
       </c>
@@ -6092,20 +6507,17 @@
       <c r="G135" s="4">
         <v>57</v>
       </c>
-      <c r="H135" s="4">
-        <v>7</v>
-      </c>
-      <c r="I135" s="4">
-        <v>7</v>
-      </c>
-      <c r="J135" s="4">
-        <v>1</v>
-      </c>
+      <c r="H135" s="4"/>
+      <c r="I135" s="4"/>
+      <c r="J135" s="4"/>
       <c r="K135" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L135" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="136" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A136" s="1" t="s">
         <v>255</v>
       </c>
@@ -6133,8 +6545,11 @@
       <c r="K136" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L136" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="137" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A137" s="1" t="s">
         <v>257</v>
       </c>
@@ -6162,8 +6577,11 @@
       <c r="K137" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L137" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="138" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A138" s="1" t="s">
         <v>259</v>
       </c>
@@ -6195,8 +6613,11 @@
       <c r="K138" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L138" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="139" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A139" s="1" t="s">
         <v>261</v>
       </c>
@@ -6228,8 +6649,11 @@
       <c r="K139" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L139" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="140" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A140" s="1" t="s">
         <v>251</v>
       </c>
@@ -6257,8 +6681,11 @@
       <c r="K140" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L140" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="141" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A141" s="1" t="s">
         <v>263</v>
       </c>
@@ -6290,8 +6717,11 @@
       <c r="K141" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L141" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="142" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A142" s="1" t="s">
         <v>265</v>
       </c>
@@ -6319,8 +6749,11 @@
       <c r="K142" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L142" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="143" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A143" s="1" t="s">
         <v>267</v>
       </c>
@@ -6352,8 +6785,11 @@
       <c r="K143" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L143" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="144" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A144" s="1" t="s">
         <v>269</v>
       </c>
@@ -6387,8 +6823,11 @@
       <c r="K144" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L144" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="145" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A145" s="1" t="s">
         <v>271</v>
       </c>
@@ -6420,8 +6859,11 @@
       <c r="K145" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L145" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="146" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A146" s="1" t="s">
         <v>273</v>
       </c>
@@ -6453,8 +6895,11 @@
       <c r="K146" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L146" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="147" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A147" s="1" t="s">
         <v>275</v>
       </c>
@@ -6486,8 +6931,11 @@
       <c r="K147" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L147" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="148" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A148" s="1" t="s">
         <v>277</v>
       </c>
@@ -6519,8 +6967,11 @@
       <c r="K148" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L148" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="149" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A149" s="1" t="s">
         <v>279</v>
       </c>
@@ -6552,8 +7003,11 @@
       <c r="K149" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L149" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="150" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A150" s="1" t="s">
         <v>281</v>
       </c>
@@ -6585,8 +7039,11 @@
       <c r="K150" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L150" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="151" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A151" s="1" t="s">
         <v>283</v>
       </c>
@@ -6614,8 +7071,11 @@
       <c r="K151" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L151" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="152" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A152" s="1" t="s">
         <v>285</v>
       </c>
@@ -6647,8 +7107,11 @@
       <c r="K152" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L152" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="153" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A153" s="1" t="s">
         <v>287</v>
       </c>
@@ -6680,8 +7143,11 @@
       <c r="K153" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L153" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="154" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A154" s="1" t="s">
         <v>289</v>
       </c>
@@ -6713,8 +7179,11 @@
       <c r="K154" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="155" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L154" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="155" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A155" s="1" t="s">
         <v>293</v>
       </c>
@@ -6746,8 +7215,11 @@
       <c r="K155" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L155" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="156" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A156" s="1" t="s">
         <v>291</v>
       </c>
@@ -6775,8 +7247,11 @@
       <c r="K156" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L156" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="157" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A157" s="1" t="s">
         <v>295</v>
       </c>
@@ -6804,8 +7279,11 @@
       <c r="K157" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="158" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L157" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="158" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A158" s="1" t="s">
         <v>297</v>
       </c>
@@ -6833,8 +7311,11 @@
       <c r="K158" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="159" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L158" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="159" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A159" s="1" t="s">
         <v>299</v>
       </c>
@@ -6862,8 +7343,11 @@
       <c r="K159" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="160" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L159" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="160" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A160" s="1" t="s">
         <v>301</v>
       </c>
@@ -6895,8 +7379,11 @@
       <c r="K160" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L160" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="161" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A161" s="1" t="s">
         <v>59</v>
       </c>
@@ -6928,8 +7415,11 @@
       <c r="K161" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L161" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="162" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A162" s="1" t="s">
         <v>303</v>
       </c>
@@ -6961,8 +7451,11 @@
       <c r="K162" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L162" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="163" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A163" s="1" t="s">
         <v>305</v>
       </c>
@@ -6994,8 +7487,11 @@
       <c r="K163" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L163" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="164" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A164" s="1" t="s">
         <v>430</v>
       </c>
@@ -7027,8 +7523,11 @@
       <c r="K164" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L164" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="165" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A165" s="1" t="s">
         <v>307</v>
       </c>
@@ -7060,8 +7559,11 @@
       <c r="K165" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L165" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="166" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A166" s="1" t="s">
         <v>309</v>
       </c>
@@ -7093,8 +7595,11 @@
       <c r="K166" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L166" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="167" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A167" s="1" t="s">
         <v>311</v>
       </c>
@@ -7126,8 +7631,11 @@
       <c r="K167" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="168" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L167" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="168" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A168" s="1" t="s">
         <v>61</v>
       </c>
@@ -7155,8 +7663,11 @@
       <c r="K168" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="169" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L168" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="169" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A169" s="1" t="s">
         <v>313</v>
       </c>
@@ -7184,8 +7695,11 @@
       <c r="K169" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="170" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L169" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="170" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A170" s="1" t="s">
         <v>315</v>
       </c>
@@ -7219,8 +7733,11 @@
       <c r="K170" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="171" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L170" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="171" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A171" s="1" t="s">
         <v>317</v>
       </c>
@@ -7252,8 +7769,11 @@
       <c r="K171" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="172" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L171" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="172" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A172" s="1" t="s">
         <v>319</v>
       </c>
@@ -7285,8 +7805,11 @@
       <c r="K172" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="173" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L172" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="173" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A173" s="1" t="s">
         <v>321</v>
       </c>
@@ -7318,8 +7841,11 @@
       <c r="K173" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="174" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L173" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="174" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A174" s="1" t="s">
         <v>424</v>
       </c>
@@ -7348,8 +7874,11 @@
       <c r="K174" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="175" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L174" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="175" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A175" s="1" t="s">
         <v>323</v>
       </c>
@@ -7381,8 +7910,11 @@
       <c r="K175" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="176" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L175" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="176" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A176" s="1" t="s">
         <v>325</v>
       </c>
@@ -7414,8 +7946,11 @@
       <c r="K176" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="177" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L176" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="177" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A177" s="1" t="s">
         <v>327</v>
       </c>
@@ -7447,8 +7982,11 @@
       <c r="K177" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="178" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L177" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="178" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A178" s="1" t="s">
         <v>329</v>
       </c>
@@ -7480,8 +8018,11 @@
       <c r="K178" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="179" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L178" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="179" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A179" s="1" t="s">
         <v>331</v>
       </c>
@@ -7513,8 +8054,11 @@
       <c r="K179" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="180" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L179" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="180" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A180" s="1" t="s">
         <v>333</v>
       </c>
@@ -7546,8 +8090,11 @@
       <c r="K180" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="181" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L180" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="181" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A181" s="1" t="s">
         <v>335</v>
       </c>
@@ -7575,8 +8122,11 @@
       <c r="K181" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="182" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L181" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="182" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A182" s="1" t="s">
         <v>337</v>
       </c>
@@ -7608,8 +8158,11 @@
       <c r="K182" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="183" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L182" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="183" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A183" s="1" t="s">
         <v>339</v>
       </c>
@@ -7637,8 +8190,11 @@
       <c r="K183" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="184" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L183" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="184" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A184" s="1" t="s">
         <v>341</v>
       </c>
@@ -7666,8 +8222,11 @@
       <c r="K184" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="185" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L184" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="185" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A185" s="1" t="s">
         <v>63</v>
       </c>
@@ -7699,8 +8258,11 @@
       <c r="K185" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="186" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L185" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="186" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A186" s="1" t="s">
         <v>343</v>
       </c>
@@ -7732,8 +8294,11 @@
       <c r="K186" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="187" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L186" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="187" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A187" s="1" t="s">
         <v>345</v>
       </c>
@@ -7761,8 +8326,11 @@
       <c r="K187" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="188" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L187" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="188" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A188" s="1" t="s">
         <v>347</v>
       </c>
@@ -7794,8 +8362,11 @@
       <c r="K188" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="189" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L188" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="189" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A189" s="1" t="s">
         <v>349</v>
       </c>
@@ -7827,8 +8398,11 @@
       <c r="K189" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="190" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L189" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="190" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A190" s="1" t="s">
         <v>351</v>
       </c>
@@ -7856,8 +8430,11 @@
       <c r="K190" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="191" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L190" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="191" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A191" s="1" t="s">
         <v>353</v>
       </c>
@@ -7889,8 +8466,11 @@
       <c r="K191" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="192" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L191" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="192" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A192" s="1" t="s">
         <v>355</v>
       </c>
@@ -7922,8 +8502,11 @@
       <c r="K192" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="193" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L192" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="193" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A193" s="1" t="s">
         <v>357</v>
       </c>
@@ -7955,8 +8538,11 @@
       <c r="K193" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="194" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L193" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="194" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A194" s="1" t="s">
         <v>359</v>
       </c>
@@ -7988,8 +8574,11 @@
       <c r="K194" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="195" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L194" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="195" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A195" s="1" t="s">
         <v>361</v>
       </c>
@@ -8021,8 +8610,11 @@
       <c r="K195" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="196" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L195" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="196" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A196" s="1" t="s">
         <v>363</v>
       </c>
@@ -8050,8 +8642,11 @@
       <c r="K196" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="197" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L196" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="197" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A197" s="1" t="s">
         <v>365</v>
       </c>
@@ -8083,8 +8678,11 @@
       <c r="K197" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="198" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L197" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="198" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A198" s="1" t="s">
         <v>367</v>
       </c>
@@ -8116,8 +8714,11 @@
       <c r="K198" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="199" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L198" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="199" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A199" s="1" t="s">
         <v>426</v>
       </c>
@@ -8142,8 +8743,11 @@
       <c r="K199" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="200" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L199" s="4" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="200" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A200" s="1" t="s">
         <v>369</v>
       </c>
@@ -8171,8 +8775,11 @@
       <c r="K200" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="201" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L200" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="201" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A201" s="1" t="s">
         <v>371</v>
       </c>
@@ -8204,8 +8811,11 @@
       <c r="K201" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="202" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L201" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="202" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A202" s="1" t="s">
         <v>65</v>
       </c>
@@ -8237,8 +8847,11 @@
       <c r="K202" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="203" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L202" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="203" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A203" s="1" t="s">
         <v>373</v>
       </c>
@@ -8266,8 +8879,11 @@
       <c r="K203" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="204" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L203" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="204" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A204" s="1" t="s">
         <v>67</v>
       </c>
@@ -8295,8 +8911,11 @@
       <c r="K204" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="205" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L204" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="205" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A205" s="1" t="s">
         <v>375</v>
       </c>
@@ -8328,8 +8947,11 @@
       <c r="K205" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="206" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L205" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="206" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A206" s="1" t="s">
         <v>377</v>
       </c>
@@ -8357,8 +8979,11 @@
       <c r="K206" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="207" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L206" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="207" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A207" s="1" t="s">
         <v>379</v>
       </c>
@@ -8386,8 +9011,11 @@
       <c r="K207" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="208" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L207" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="208" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A208" s="1" t="s">
         <v>381</v>
       </c>
@@ -8419,8 +9047,11 @@
       <c r="K208" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="209" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L208" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="209" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A209" s="1" t="s">
         <v>383</v>
       </c>
@@ -8452,8 +9083,11 @@
       <c r="K209" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="210" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L209" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="210" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A210" s="1" t="s">
         <v>385</v>
       </c>
@@ -8485,8 +9119,11 @@
       <c r="K210" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="211" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L210" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="211" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A211" s="1" t="s">
         <v>387</v>
       </c>
@@ -8518,8 +9155,11 @@
       <c r="K211" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="212" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L211" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="212" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A212" s="1" t="s">
         <v>389</v>
       </c>
@@ -8553,8 +9193,11 @@
       <c r="K212" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="213" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L212" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="213" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A213" s="1" t="s">
         <v>391</v>
       </c>
@@ -8588,8 +9231,11 @@
       <c r="K213" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="214" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L213" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="214" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A214" s="1" t="s">
         <v>393</v>
       </c>
@@ -8621,8 +9267,11 @@
       <c r="K214" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="215" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L214" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="215" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A215" s="1" t="s">
         <v>395</v>
       </c>
@@ -8654,8 +9303,11 @@
       <c r="K215" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="216" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L215" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="216" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A216" s="1" t="s">
         <v>397</v>
       </c>
@@ -8687,8 +9339,11 @@
       <c r="K216" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="217" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L216" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="217" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A217" s="1" t="s">
         <v>399</v>
       </c>
@@ -8720,8 +9375,11 @@
       <c r="K217" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="218" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L217" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="218" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A218" s="1" t="s">
         <v>401</v>
       </c>
@@ -8753,8 +9411,11 @@
       <c r="K218" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="219" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L218" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="219" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A219" s="1" t="s">
         <v>403</v>
       </c>
@@ -8786,8 +9447,11 @@
       <c r="K219" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="220" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L219" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="220" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A220" s="1" t="s">
         <v>405</v>
       </c>
@@ -8821,13 +9485,16 @@
       <c r="K220" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="221" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L220" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="221" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A221" s="1" t="s">
         <v>407</v>
       </c>
       <c r="B221" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="C221">
         <v>3</v>
@@ -8854,10 +9521,13 @@
       <c r="K221" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="222" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L221" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="222" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B222" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="G222" s="4">
         <v>67</v>
@@ -8868,8 +9538,11 @@
       <c r="K222" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="223" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L222" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="223" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A223" s="1" t="s">
         <v>69</v>
       </c>
@@ -8897,8 +9570,11 @@
       <c r="K223" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="224" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L223" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="224" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A224" s="1" t="s">
         <v>408</v>
       </c>
@@ -8930,8 +9606,11 @@
       <c r="K224" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="225" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L224" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="225" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A225" s="1" t="s">
         <v>412</v>
       </c>
@@ -8963,8 +9642,11 @@
       <c r="K225" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="226" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L225" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="226" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A226" s="1" t="s">
         <v>410</v>
       </c>
@@ -8996,8 +9678,11 @@
       <c r="K226" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="227" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L226" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="227" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A227" s="1" t="s">
         <v>414</v>
       </c>
@@ -9029,8 +9714,11 @@
       <c r="K227" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="228" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L227" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="228" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A228" s="1" t="s">
         <v>416</v>
       </c>
@@ -9058,8 +9746,11 @@
       <c r="K228" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="229" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L228" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="229" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A229" s="1" t="s">
         <v>418</v>
       </c>
@@ -9087,8 +9778,11 @@
       <c r="K229" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="230" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L229" s="4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="230" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A230" s="1" t="s">
         <v>420</v>
       </c>
@@ -9116,31 +9810,9 @@
       <c r="K230" s="4">
         <v>3</v>
       </c>
-    </row>
-    <row r="231" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A231" s="1" t="s">
-        <v>440</v>
-      </c>
-      <c r="B231" t="s">
-        <v>441</v>
-      </c>
-      <c r="C231">
-        <v>2</v>
-      </c>
-      <c r="D231">
-        <v>4</v>
-      </c>
-      <c r="E231">
-        <v>4</v>
-      </c>
-      <c r="F231">
-        <v>0</v>
-      </c>
-      <c r="G231" s="4"/>
-      <c r="H231" s="4"/>
-      <c r="I231" s="4"/>
-      <c r="J231" s="4"/>
-      <c r="K231" s="4"/>
+      <c r="L230" s="4" t="s">
+        <v>464</v>
+      </c>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0"/>

</xml_diff>